<commit_message>
DATA: sync 9 new records (total 48)
</commit_message>
<xml_diff>
--- a/QA_Defects_Data.xlsx
+++ b/QA_Defects_Data.xlsx
@@ -1,12 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -49,7 +50,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -412,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,7 +461,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-31 00:00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -493,14 +494,14 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Surface scratch found on outer diameter</t>
+          <t>Surface scratch on outer diameter</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-01 00:00:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -533,64 +534,64 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Dent mark on corner area</t>
+          <t>Dent mark on corner</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-09-02 00:00:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BTD</t>
+          <t>KSV</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>PLASTIC</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PART MISTAKE</t>
+          <t>LEAK</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>COVER HOUSING</t>
+          <t>CAPACITOR 450V</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4P022001-2 B</t>
+          <t>VE101-22A</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Wrong color delivered (Black vs Grey)</t>
+          <t>Insulation damage detected</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-09-03 00:00:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>C.G.</t>
+          <t>AKUSAN</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SEALING</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -600,277 +601,277 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>O-RING 25.4MM</t>
+          <t>CONNECTOR 2PIN</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>5P100105-1</t>
+          <t>AC2019-A</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Deformation found at joint area</t>
+          <t>Pin misalignment</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-09-04 00:00:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TTS PLASTIC</t>
+          <t>BTD</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>PACKING</t>
+          <t>PLASTIC</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>PART MISTAKE</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>FOAM PACKING</t>
+          <t>COVER HOUSING</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>6P200450-1</t>
+          <t>4P022001-2 B</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Thickness out of spec</t>
+          <t>Wrong color (Black vs Grey)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-09-10 00:00:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KSV</t>
+          <t>BTD</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>PLASTIC</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>LEAK</t>
+          <t>PART MISTAKE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CAPACITOR 450V</t>
+          <t>COVER HOUSING</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>VE101-22A</t>
+          <t>4P022001-2 B</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>12</v>
+        <v>600</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Insulation damage detected</t>
+          <t>Wrong color (Black vs Grey)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-09-11 00:00:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AKUSAN</t>
+          <t>BTD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>PLASTIC</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>PART MISTAKE</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>CONNECTOR 2PIN</t>
+          <t>COVER HOUSING</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AC2019-A</t>
+          <t>4P022001-2 B</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>8</v>
+        <v>700</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Pin misalignment</t>
+          <t>Wrong color (Black vs Grey)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-12 00:00:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NISSEN CHEMITEC</t>
+          <t>BTD</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>PIPING</t>
+          <t>PLASTIC</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>LEAK</t>
+          <t>PART MISTAKE</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>PIPE JOINT</t>
+          <t>COVER HOUSING</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1P095005-2 K</t>
+          <t>4P022001-2 B</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>15</v>
+        <v>800</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Thread gap exceeds tolerance</t>
+          <t>Wrong color (Black vs Grey)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-09-13 00:00:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PARADISE</t>
+          <t>BTD</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SHEET METAL</t>
+          <t>PLASTIC</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FUNCTION NG</t>
+          <t>PART MISTAKE</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BRACKET L</t>
+          <t>COVER HOUSING</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>3P811369-1 A</t>
+          <t>4P022001-2 B</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>3</v>
+        <v>900</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Bending angle incorrect</t>
+          <t>Wrong color (Black vs Grey)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SAMBO</t>
+          <t>NISSEN CHEMITEC</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PLASTIC</t>
+          <t>PIPING</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DIMENSION NG</t>
+          <t>APPEARANCE NG</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>COVER A</t>
+          <t>ELBOW PIPE 1/2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>7P033110-1</t>
+          <t>1P095004-1 K</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>5</v>
+        <v>120</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Dimension 0.3mm out of spec</t>
+          <t>Surface scratch found on outer diameter</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>KSV</t>
+          <t>PARADISE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>SHEET METAL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -880,77 +881,77 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>RESISTOR 10K</t>
+          <t>INSTALLATION PLATE</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>VE100-12B</t>
+          <t>3P811368-1 A</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>9</v>
+        <v>51</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Color code wrong</t>
+          <t>Dent mark on corner area</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>BTD</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>PLASTIC</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>PART MISTAKE</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PCB ASSY POWER</t>
+          <t>COVER HOUSING</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>EX30037-P</t>
+          <t>4P022001-2 B</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Assemble L2R reverse</t>
+          <t>Wrong color delivered (Black vs Grey)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>APT (Thailand)</t>
+          <t>C.G.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>SEALING</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -960,37 +961,37 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>ACCUMULATOR ASSY</t>
+          <t>O-RING 25.4MM</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2969059</t>
+          <t>5P100105-1</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Lead wire has notch mark</t>
+          <t>Deformation found at joint area</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PARADISE</t>
+          <t>TTS PLASTIC</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>PACKING</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1000,192 +1001,192 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>COMPRESSOR</t>
+          <t>FOAM PACKING</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2969059</t>
+          <t>6P200450-1</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Lead wire has notch mark</t>
+          <t>Thickness out of spec</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SUPERFAST</t>
+          <t>KSV</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RUBBER</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>LEAK</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>GASKET 50MM</t>
+          <t>CAPACITOR 450V</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>8P044001-1</t>
+          <t>VE101-22A</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Surface contamination</t>
+          <t>Insulation damage detected</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SAM NEO</t>
+          <t>AKUSAN</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>RAW MATERIAL</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>FUNCTION NG</t>
+          <t>APPEARANCE NG</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RAW RESIN</t>
+          <t>CONNECTOR 2PIN</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>9P055002-1</t>
+          <t>AC2019-A</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Hardness not meeting spec</t>
+          <t>Pin misalignment</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TECHNO ASSOCIATE</t>
+          <t>NISSEN CHEMITEC</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PRINTING</t>
+          <t>PIPING</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>PART MISTAKE</t>
+          <t>LEAK</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LABEL STICKER</t>
+          <t>PIPE JOINT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>10P066003-1</t>
+          <t>1P095005-2 K</t>
         </is>
       </c>
       <c r="G18" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Wrong label printed</t>
+          <t>Thread gap exceeds tolerance</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>NISSEN CHEMITEC</t>
+          <t>PARADISE</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PIPING</t>
+          <t>SHEET METAL</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>FUNCTION NG</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ELBOW PIPE 3/4</t>
+          <t>BRACKET L</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1P095006-1 K</t>
+          <t>3P811369-1 A</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Surface scratch found</t>
+          <t>Bending angle incorrect</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BTD</t>
+          <t>SAMBO</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1200,27 +1201,27 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>HOUSING B</t>
+          <t>COVER A</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>4P022002-2 B</t>
+          <t>7P033110-1</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Dimension 0.5mm out of spec</t>
+          <t>Dimension 0.3mm out of spec</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1235,37 +1236,37 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>LEAK</t>
+          <t>APPEARANCE NG</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CONNECTOR 3PIN</t>
+          <t>RESISTOR 10K</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>VE102-33C</t>
+          <t>VE100-12B</t>
         </is>
       </c>
       <c r="G21" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Seal failure detected</t>
+          <t>Color code wrong</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PARADISE</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1280,12 +1281,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>COMPRESSOR</t>
+          <t>PCB ASSY POWER</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2969059</t>
+          <t>EX30037-P</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1293,14 +1294,14 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Lead wire has notch mark</t>
+          <t>Assemble L2R reverse</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1310,42 +1311,42 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>RAW MATERIAL</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>FUNCTION NG</t>
+          <t>APPEARANCE NG</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RAW ALUMINUM</t>
+          <t>ACCUMULATOR ASSY</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>11P077001-1</t>
+          <t>2969059</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Composition out of spec</t>
+          <t>Lead wire has notch mark</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>KSV</t>
+          <t>PARADISE</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1355,162 +1356,162 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>PART MISTAKE</t>
+          <t>APPEARANCE NG</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>IC CHIP</t>
+          <t>COMPRESSOR</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>VE103-44D</t>
+          <t>2969059</t>
         </is>
       </c>
       <c r="G24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Wrong part number</t>
+          <t>Lead wire has notch mark</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AKUSAN</t>
+          <t>SUPERFAST</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>RUBBER</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>LEAK</t>
+          <t>APPEARANCE NG</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>WIRE HARNESS</t>
+          <t>GASKET 50MM</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AC2020-B</t>
+          <t>8P044001-1</t>
         </is>
       </c>
       <c r="G25" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Loose connection</t>
+          <t>Surface contamination</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>PARADISE</t>
+          <t>SAM NEO</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SHEET METAL</t>
+          <t>RAW MATERIAL</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>DIMENSION NG</t>
+          <t>FUNCTION NG</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>BRACKET R</t>
+          <t>RAW RESIN</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>3P811370-1 A</t>
+          <t>9P055002-1</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Hole position 0.2mm off</t>
+          <t>Hardness not meeting spec</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SUPERFAST</t>
+          <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>RUBBER</t>
+          <t>PRINTING</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>PART MISTAKE</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>GASKET 60MM</t>
+          <t>LABEL STICKER</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>8P044002-1</t>
+          <t>10P066003-1</t>
         </is>
       </c>
       <c r="G27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Surface contamination</t>
+          <t>Wrong label printed</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SAMBO</t>
+          <t>NISSEN CHEMITEC</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PLASTIC</t>
+          <t>PIPING</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1520,77 +1521,77 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>COVER B</t>
+          <t>ELBOW PIPE 3/4</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>7P033111-1</t>
+          <t>1P095006-1 K</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Color inconsistency</t>
+          <t>Surface scratch found</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>TECHNO ASSOCIATE</t>
+          <t>BTD</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PRINTING</t>
+          <t>PLASTIC</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>DIMENSION NG</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>LABEL STICKER</t>
+          <t>HOUSING B</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>10P066004-1</t>
+          <t>4P022002-2 B</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Print smudge detected</t>
+          <t>Dimension 0.5mm out of spec</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>C.G.</t>
+          <t>KSV</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SEALING</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1600,187 +1601,187 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>GASKET 40MM</t>
+          <t>CONNECTOR 3PIN</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>5P100106-1</t>
+          <t>VE102-33C</t>
         </is>
       </c>
       <c r="G30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Compression set issue</t>
+          <t>Seal failure detected</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>TTS PLASTIC</t>
+          <t>PARADISE</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PACKING</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>DIMENSION NG</t>
+          <t>APPEARANCE NG</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FOAM PACKING</t>
+          <t>COMPRESSOR</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>6P200451-1</t>
+          <t>2969059</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Thickness out of spec</t>
+          <t>Lead wire has notch mark</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>NISSEN CHEMITEC</t>
+          <t>APT (Thailand)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PIPING</t>
+          <t>RAW MATERIAL</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>FUNCTION NG</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>ELBOW PIPE 1/2</t>
+          <t>RAW ALUMINUM</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1P095004-1 K</t>
+          <t>11P077001-1</t>
         </is>
       </c>
       <c r="G32" t="n">
-        <v>120</v>
+        <v>5</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Surface scratch</t>
+          <t>Composition out of spec</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-03</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PARADISE</t>
+          <t>KSV</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SHEET METAL</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>PART MISTAKE</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>INSTALLATION PLATE</t>
+          <t>IC CHIP</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>3P811368-1 A</t>
+          <t>VE103-44D</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Dent mark</t>
+          <t>Wrong part number</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>NISSEN CHEMITEC</t>
+          <t>AKUSAN</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>PIPING</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>LEAK</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>ELBOW PIPE 1/2</t>
+          <t>WIRE HARNESS</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1P095004-1 K</t>
+          <t>AC2020-B</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>120</v>
+        <v>2</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Surface scratch</t>
+          <t>Loose connection</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1795,82 +1796,82 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>DIMENSION NG</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>INSTALLATION PLATE</t>
+          <t>BRACKET R</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>3P811368-1 A</t>
+          <t>3P811370-1 A</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Dent mark</t>
+          <t>Hole position 0.2mm off</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>KSV</t>
+          <t>SUPERFAST</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>RUBBER</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LEAK</t>
+          <t>APPEARANCE NG</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>CAPACITOR 450V</t>
+          <t>GASKET 60MM</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>VE101-22A</t>
+          <t>8P044002-1</t>
         </is>
       </c>
       <c r="G36" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Insulation damage</t>
+          <t>Surface contamination</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-10</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>AKUSAN</t>
+          <t>SAMBO</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>PLASTIC</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1880,77 +1881,77 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>CONNECTOR 2PIN</t>
+          <t>COVER B</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>AC2019-A</t>
+          <t>7P033111-1</t>
         </is>
       </c>
       <c r="G37" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Pin misalignment</t>
+          <t>Color inconsistency</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>BTD</t>
+          <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PLASTIC</t>
+          <t>PRINTING</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>PART MISTAKE</t>
+          <t>APPEARANCE NG</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>COVER HOUSING</t>
+          <t>LABEL STICKER</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>4P022001-2 B</t>
+          <t>10P066004-1</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Wrong color</t>
+          <t>Print smudge detected</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>KSV</t>
+          <t>C.G.</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>SEALING</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1960,64 +1961,424 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>CAPACITOR BATCH</t>
+          <t>GASKET 40MM</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>VE101-22B</t>
+          <t>5P100106-1</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>600</v>
+        <v>3</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Batch defect</t>
+          <t>Compression set issue</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>TTS PLASTIC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PACKING</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>DIMENSION NG</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>FOAM PACKING</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>6P200451-1</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>9</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Thickness out of spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>NISSEN CHEMITEC</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PIPING</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ELBOW PIPE 1/2</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1P095004-1 K</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>120</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Surface scratch</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>PARADISE</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>SHEET METAL</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>INSTALLATION PLATE</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>3P811368-1 A</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>51</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Dent mark</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>NISSEN CHEMITEC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PIPING</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ELBOW PIPE 1/2</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>1P095004-1 K</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>120</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Surface scratch</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>PARADISE</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>SHEET METAL</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>INSTALLATION PLATE</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>3P811368-1 A</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>51</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Dent mark</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>KSV</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ELECTRIC &amp; ELEC.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>LEAK</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>CAPACITOR 450V</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>VE101-22A</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>12</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Insulation damage</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>AKUSAN</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>ELECTRIC &amp; ELEC.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>CONNECTOR 2PIN</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>AC2019-A</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>8</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Pin misalignment</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>BTD</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>PLASTIC</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>PART MISTAKE</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>COVER HOUSING</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>4P022001-2 B</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>25</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Wrong color</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>KSV</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>ELECTRIC &amp; ELEC.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>LEAK</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>CAPACITOR BATCH</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>VE101-22B</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>600</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Batch defect</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
         <is>
           <t>TEST-SYNC</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>TEST PART</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>TEST-001</t>
         </is>
       </c>
-      <c r="G40" t="n">
+      <c r="G49" t="n">
         <v>99</v>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>Sync test from local</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
DATA: sync 9 new records (dedup, total 46)
</commit_message>
<xml_diff>
--- a/QA_Defects_Data.xlsx
+++ b/QA_Defects_Data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H49"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2106,35 +2106,35 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>NISSEN CHEMITEC</t>
+          <t>KSV</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PIPING</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>LEAK</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>ELBOW PIPE 1/2</t>
+          <t>CAPACITOR 450V</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>1P095004-1 K</t>
+          <t>VE101-22A</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>120</v>
+        <v>12</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Surface scratch</t>
+          <t>Insulation damage</t>
         </is>
       </c>
     </row>
@@ -2146,12 +2146,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>PARADISE</t>
+          <t>AKUSAN</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SHEET METAL</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2161,20 +2161,20 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>INSTALLATION PLATE</t>
+          <t>CONNECTOR 2PIN</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>3P811368-1 A</t>
+          <t>AC2019-A</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>51</v>
+        <v>8</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Dent mark</t>
+          <t>Pin misalignment</t>
         </is>
       </c>
     </row>
@@ -2186,35 +2186,35 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>KSV</t>
+          <t>BTD</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ELECTRIC &amp; ELEC.</t>
+          <t>PLASTIC</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>LEAK</t>
+          <t>PART MISTAKE</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>CAPACITOR 450V</t>
+          <t>COVER HOUSING</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>VE101-22A</t>
+          <t>4P022001-2 B</t>
         </is>
       </c>
       <c r="G45" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Insulation damage</t>
+          <t>Wrong color</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>AKUSAN</t>
+          <t>KSV</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2236,25 +2236,25 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>APPEARANCE NG</t>
+          <t>LEAK</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>CONNECTOR 2PIN</t>
+          <t>CAPACITOR BATCH</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>AC2019-A</t>
+          <t>VE101-22B</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>8</v>
+        <v>600</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Pin misalignment</t>
+          <t>Batch defect</t>
         </is>
       </c>
     </row>
@@ -2266,113 +2266,33 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>BTD</t>
+          <t>TEST-SYNC</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PLASTIC</t>
+          <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>PART MISTAKE</t>
+          <t>FUNCTION NG</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>COVER HOUSING</t>
+          <t>TEST PART</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>4P022001-2 B</t>
+          <t>TEST-001</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>25</v>
+        <v>99</v>
       </c>
       <c r="H47" t="inlineStr">
-        <is>
-          <t>Wrong color</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>KSV</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>ELECTRIC &amp; ELEC.</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>LEAK</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>CAPACITOR BATCH</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>VE101-22B</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>600</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Batch defect</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2026-08-31</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>TEST-SYNC</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>ELECTRIC &amp; ELEC.</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>FUNCTION NG</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>TEST PART</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>TEST-001</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>99</v>
-      </c>
-      <c r="H49" t="inlineStr">
         <is>
           <t>Sync test from local</t>
         </is>

</xml_diff>

<commit_message>
DATA: sync 37 new records (dedup, total 92)
</commit_message>
<xml_diff>
--- a/QA_Defects_Data.xlsx
+++ b/QA_Defects_Data.xlsx
@@ -1,14 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defects Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,48 +25,16 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00B71C1C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFD700"/>
-        <bgColor rgb="00FFD700"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF8DC"/>
-        <bgColor rgb="00FFF8DC"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -75,39 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="00000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="00000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00000000"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -473,2431 +413,3729 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:H93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="35" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Group Part</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Problem Mode</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Part Name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Part No</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>AKUSAN</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SHEET METAL</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>DIMENSION NG</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>GASKET RING</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>PAR-001</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>120</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Surface scratch found on outer diameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AKUSAN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SEALING</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FUNCTION NG</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>PIPE CONNECTOR</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>VE100-15B</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Wrong part shipped - mismatch with PO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PARADISE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>RUBBER</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>LEAK</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ELBOW PIPE 1/2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>VE101-22A</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>50</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Dimensional out of spec by 0.2mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SAMBO</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>PIPING</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>LEAK</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>O-RING SEAL</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>AC2019-A</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Color mismatch with sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>KSV</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PLASTIC</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>HOSE CLAMP</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>AC2020-B</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Color mismatch with sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PARADISE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SHEET METAL</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>PART MISTAKE</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>GASKET RING</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PAR-001</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Color mismatch with sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SAMBO</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ELECTRIC &amp; ELEC.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>FUNCTION NG</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>O-RING SEAL</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>AC2019-A</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>50</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Surface scratch found on outer diameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AKUSAN</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>PACKING</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>FUNCTION NG</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>VALVE BODY</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PAR-002</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>8</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Dimensional out of spec by 0.2mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>C.G.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>RUBBER</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>FUNCTION NG</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PIPE CONNECTOR</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>VE100-15B</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>120</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Color mismatch with sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TTS PLASTIC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SEALING</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>HOSE CLAMP</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>AC2020-B</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>120</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Color mismatch with sample</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PARADISE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>RAW MATERIAL</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>PART MISTAKE</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>VALVE BODY</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PAR-002</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Function test failed - leakage detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AKUSAN</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SEALING</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>LEAK</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>HEAT SHRINK</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>NS-CHEM-002</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>120</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Dimensional out of spec by 0.2mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>TTS PLASTIC</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>RAW MATERIAL</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>LEAK</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>TERMINAL BLOCK</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>NS-CHEM-001</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>50</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Surface contamination visible</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TTS PLASTIC</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>RAW MATERIAL</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PIPE CONNECTOR</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>VE100-15B</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Wrong part shipped - mismatch with PO</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>NISSEN CHEMITEC</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SEALING</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>LEAK</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>GASKET RING</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PAR-001</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Crack visible at weld joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>AKUSAN</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>RUBBER</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>DIMENSION NG</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PIPE CONNECTOR</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>VE100-15B</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Surface scratch found on outer diameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>PARADISE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SHEET METAL</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>LEAK</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>VALVE BODY</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PAR-002</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Surface contamination visible</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>TTS PLASTIC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>RUBBER</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PIPE CONNECTOR</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>VE100-15B</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>12</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Function test failed - leakage detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>NISSEN CHEMITEC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>PACKING</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>DIMENSION NG</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>TERMINAL BLOCK</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>NS-CHEM-001</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>25</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Dimensional out of spec by 0.2mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>KSV</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ELECTRIC &amp; ELEC.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>TERMINAL BLOCK</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>VE101-22A</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>250</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Major defect - entire batch rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>PARADISE</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>RUBBER</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PIPE CONNECTOR</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>VE100-15B</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Dimensional out of spec by 0.2mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>AKUSAN</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ELECTRIC &amp; ELEC.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FUNCTION NG</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>HOSE CLAMP</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>AC2020-B</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Dimensional out of spec by 0.2mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>AKUSAN</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PIPING</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>LEAK</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>GASKET RING</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>PAR-001</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Surface scratch found on outer diameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TTS PLASTIC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>RUBBER</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>PART MISTAKE</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>TERMINAL BLOCK</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>NS-CHEM-001</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Surface contamination visible</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>AKUSAN</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ELECTRIC &amp; ELEC.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>DIMENSION NG</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>TERMINAL BLOCK</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>NS-CHEM-001</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Surface contamination visible</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>PARADISE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>PLASTIC</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>HOSE CLAMP</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>AC2020-B</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Surface contamination visible</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>C.G.</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PIPING</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>DIMENSION NG</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>HOSE CLAMP</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>AC2020-B</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>3</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Crack visible at weld joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>NISSEN CHEMITEC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PACKING</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>FUNCTION NG</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>TERMINAL BLOCK</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>NS-CHEM-001</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Dimensional out of spec by 0.2mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>C.G.</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>PIPING</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>GASKET RING</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>PAR-001</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Function test failed - leakage detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>KSV</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>PLASTIC</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>PART MISTAKE</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>ELBOW PIPE 1/2</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>VE101-22A</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Function test failed - leakage detected</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>PARADISE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>SEALING</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PART MISTAKE</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>HEAT SHRINK</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>NS-CHEM-002</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>25</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Crack visible at weld joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>C.G.</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>SEALING</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>VALVE BODY</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>PAR-002</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>50</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Surface scratch found on outer diameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>BTD</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>RUBBER</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>DIMENSION NG</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>HEAT SHRINK</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>NS-CHEM-002</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Crack visible at weld joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>BTD</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>RUBBER</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>HOSE CLAMP</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>AC2020-B</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>120</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Surface scratch found on outer diameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-19 00:00:00</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>BTD</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>RUBBER</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>APPEARANCE NG</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>HOSE CLAMP</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>AC2020-B</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>600</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Surface scratch found on outer diameter</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
         <is>
           <t>NISSEN</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>SL-50</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G37" t="n">
         <v>5</v>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be SL-75</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>VE102-33C</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G38" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>Battery Cell Holder dimension out of spec by 0.2mm</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>PL-2020</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G39" t="n">
         <v>11</v>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>CASE - LED Indicator dimension out of spec by 0.2mm (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>KSV</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>SM-A1</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G40" t="n">
         <v>6</v>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>Color mismatch vs Pantone reference</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>RB-100</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G41" t="n">
         <v>16</v>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>Surface scratch on gasket ring</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>APT</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="G42" t="n">
         <v>8</v>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>CASE - Color mismatch vs Pantone reference (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>PL-2020</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G43" t="n">
         <v>23</v>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>Visible defect on terminal block surface</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>Cover Cap</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>P-101</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="G44" t="n">
         <v>24</v>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>CASE - Cover Cap function test failed (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>PK-001</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="G45" t="n">
         <v>5</v>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be PK-001</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>PK-002</t>
         </is>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="G46" t="n">
         <v>4</v>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>Main Board dimension out of spec by 0.2mm</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>PK-001</t>
         </is>
       </c>
-      <c r="G12" s="3" t="n">
+      <c r="G47" t="n">
         <v>17</v>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>CASE - Gasket Ring dimension out of spec by 0.2mm (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+    <row r="48">
+      <c r="A48" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>RB-100</t>
         </is>
       </c>
-      <c r="G13" s="3" t="n">
+      <c r="G48" t="n">
         <v>17</v>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H48" t="inlineStr">
         <is>
           <t>Surface scratch on switch button</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>VE103-44D</t>
         </is>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="G49" t="n">
         <v>20</v>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be VE100-15C</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="50">
+      <c r="A50" t="inlineStr">
         <is>
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>VE100-15C</t>
         </is>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="G50" t="n">
         <v>25</v>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>Visible defect on led indicator surface</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>VE100-15C</t>
         </is>
       </c>
-      <c r="G16" s="3" t="n">
+      <c r="G51" t="n">
         <v>6</v>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>Visible defect on switch button surface</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+    <row r="52">
+      <c r="A52" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>SURFACE DEFECT</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>RM-A</t>
         </is>
       </c>
-      <c r="G17" s="3" t="n">
+      <c r="G52" t="n">
         <v>19</v>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>Surface scratch on switch button</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>PRINTING</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>PR-BARCODE</t>
         </is>
       </c>
-      <c r="G18" s="3" t="n">
+      <c r="G53" t="n">
         <v>4</v>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>LED Indicator leak detected at joint</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>VE103-44D</t>
         </is>
       </c>
-      <c r="G19" s="3" t="n">
+      <c r="G54" t="n">
         <v>23</v>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>Gasket Ring dimension out of spec by 0.2mm</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>Cable Harness</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>RB-200</t>
         </is>
       </c>
-      <c r="G20" s="3" t="n">
+      <c r="G55" t="n">
         <v>9</v>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H55" t="inlineStr">
         <is>
           <t>Color mismatch vs Pantone reference</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>SAM NEO</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>RM-B</t>
         </is>
       </c>
-      <c r="G21" s="3" t="n">
+      <c r="G56" t="n">
         <v>2</v>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H56" t="inlineStr">
         <is>
           <t>CASE - Gasket Ring leak detected at joint (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="57">
+      <c r="A57" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>SM-A1</t>
         </is>
       </c>
-      <c r="G22" s="3" t="n">
+      <c r="G57" t="n">
         <v>14</v>
       </c>
-      <c r="H22" s="3" t="inlineStr">
+      <c r="H57" t="inlineStr">
         <is>
           <t>Switch Button function test failed</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Cover Cap</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>PL-2020</t>
         </is>
       </c>
-      <c r="G23" s="3" t="n">
+      <c r="G58" t="n">
         <v>15</v>
       </c>
-      <c r="H23" s="3" t="inlineStr">
+      <c r="H58" t="inlineStr">
         <is>
           <t>Cover Cap function test failed</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="59">
+      <c r="A59" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>SAM NEO</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>COLOR NG</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>VE101-22A</t>
         </is>
       </c>
-      <c r="G24" s="3" t="n">
+      <c r="G59" t="n">
         <v>22</v>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H59" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be VE102-33C</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="60">
+      <c r="A60" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B60" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="F60" t="inlineStr">
         <is>
           <t>PK-001</t>
         </is>
       </c>
-      <c r="G25" s="3" t="n">
+      <c r="G60" t="n">
         <v>24</v>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H60" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be PK-001</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>KSV</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>PRINTING</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>PR-LABEL</t>
         </is>
       </c>
-      <c r="G26" s="3" t="n">
+      <c r="G61" t="n">
         <v>22</v>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H61" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be PR-LABEL</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="62">
+      <c r="A62" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B62" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D62" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G27" s="3" t="n">
+      <c r="G62" t="n">
         <v>12</v>
       </c>
-      <c r="H27" s="3" t="inlineStr">
+      <c r="H62" t="inlineStr">
         <is>
           <t>Visible defect on terminal block surface</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>SM-A1</t>
         </is>
       </c>
-      <c r="G28" s="3" t="n">
+      <c r="G63" t="n">
         <v>24</v>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H63" t="inlineStr">
         <is>
           <t>CASE - Main Board dimension out of spec by 0.2mm (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="64">
+      <c r="A64" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G29" s="3" t="n">
+      <c r="G64" t="n">
         <v>16</v>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="H64" t="inlineStr">
         <is>
           <t>CASE - Battery Cell Holder leak detected at joint (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B65" t="inlineStr">
         <is>
           <t>C.G.</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>RM-A</t>
         </is>
       </c>
-      <c r="G30" s="3" t="n">
+      <c r="G65" t="n">
         <v>11</v>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="H65" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be RM-B</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G31" s="3" t="n">
+      <c r="G66" t="n">
         <v>17</v>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="H66" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be SL-75</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D67" t="inlineStr">
         <is>
           <t>COLOR NG</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E67" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>PK-002</t>
         </is>
       </c>
-      <c r="G32" s="3" t="n">
+      <c r="G67" t="n">
         <v>4</v>
       </c>
-      <c r="H32" s="3" t="inlineStr">
+      <c r="H67" t="inlineStr">
         <is>
           <t>Color mismatch vs Pantone reference</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="68">
+      <c r="A68" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D68" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E68" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F68" t="inlineStr">
         <is>
           <t>VE100-15C</t>
         </is>
       </c>
-      <c r="G33" s="3" t="n">
+      <c r="G68" t="n">
         <v>4</v>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H68" t="inlineStr">
         <is>
           <t>CASE - Color mismatch vs Pantone reference (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B69" t="inlineStr">
         <is>
           <t>SAM NEO</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D69" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>P-330</t>
         </is>
       </c>
-      <c r="G34" s="3" t="n">
+      <c r="G69" t="n">
         <v>7</v>
       </c>
-      <c r="H34" s="3" t="inlineStr">
+      <c r="H69" t="inlineStr">
         <is>
           <t>Visible defect on battery cell holder surface</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="70">
+      <c r="A70" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B70" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>RM-A</t>
         </is>
       </c>
-      <c r="G35" s="3" t="n">
+      <c r="G70" t="n">
         <v>22</v>
       </c>
-      <c r="H35" s="3" t="inlineStr">
+      <c r="H70" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be RM-A</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="71">
+      <c r="A71" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E71" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>P-330</t>
         </is>
       </c>
-      <c r="G36" s="3" t="n">
+      <c r="G71" t="n">
         <v>10</v>
       </c>
-      <c r="H36" s="3" t="inlineStr">
+      <c r="H71" t="inlineStr">
         <is>
           <t>Main Board leak detected at joint</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="72">
+      <c r="A72" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="B72" t="inlineStr">
         <is>
           <t>NISSEN</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t>Cover Cap</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>RB-100</t>
         </is>
       </c>
-      <c r="G37" s="3" t="n">
+      <c r="G72" t="n">
         <v>12</v>
       </c>
-      <c r="H37" s="3" t="inlineStr">
+      <c r="H72" t="inlineStr">
         <is>
           <t>Visible defect on cover cap surface</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="73">
+      <c r="A73" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G38" s="3" t="n">
+      <c r="G73" t="n">
         <v>14</v>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="H73" t="inlineStr">
         <is>
           <t>CASE - Terminal Block dimension out of spec by 0.2mm (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="74">
+      <c r="A74" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B74" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>PRINTING</t>
         </is>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>PR-BARCODE</t>
         </is>
       </c>
-      <c r="G39" s="3" t="n">
+      <c r="G74" t="n">
         <v>6</v>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="H74" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be PR-LABEL</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="75">
+      <c r="A75" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>RB-200</t>
         </is>
       </c>
-      <c r="G40" s="3" t="n">
+      <c r="G75" t="n">
         <v>13</v>
       </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="H75" t="inlineStr">
         <is>
           <t>CASE - Surface scratch on switch button (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="76">
+      <c r="A76" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B76" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>Cable Harness</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>P-205</t>
         </is>
       </c>
-      <c r="G41" s="3" t="n">
+      <c r="G76" t="n">
         <v>3</v>
       </c>
-      <c r="H41" s="3" t="inlineStr">
+      <c r="H76" t="inlineStr">
         <is>
           <t>Surface scratch on cable harness</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="77">
+      <c r="A77" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D77" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>Cable Harness</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>PK-001</t>
         </is>
       </c>
-      <c r="G42" s="3" t="n">
+      <c r="G77" t="n">
         <v>4</v>
       </c>
-      <c r="H42" s="3" t="inlineStr">
+      <c r="H77" t="inlineStr">
         <is>
           <t>Visible defect on cable harness surface</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+    <row r="78">
+      <c r="A78" t="inlineStr">
         <is>
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D78" t="inlineStr">
         <is>
           <t>COLOR NG</t>
         </is>
       </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>Cable Harness</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F78" t="inlineStr">
         <is>
           <t>RM-A</t>
         </is>
       </c>
-      <c r="G43" s="3" t="n">
+      <c r="G78" t="n">
         <v>22</v>
       </c>
-      <c r="H43" s="3" t="inlineStr">
+      <c r="H78" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be RM-A</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+    <row r="79">
+      <c r="A79" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E79" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F79" t="inlineStr">
         <is>
           <t>PL-2019</t>
         </is>
       </c>
-      <c r="G44" s="3" t="n">
+      <c r="G79" t="n">
         <v>19</v>
       </c>
-      <c r="H44" s="3" t="inlineStr">
+      <c r="H79" t="inlineStr">
         <is>
           <t>Color mismatch vs Pantone reference</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+    <row r="80">
+      <c r="A80" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="B80" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="E80" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F80" t="inlineStr">
         <is>
           <t>VE101-22A</t>
         </is>
       </c>
-      <c r="G45" s="3" t="n">
+      <c r="G80" t="n">
         <v>13</v>
       </c>
-      <c r="H45" s="4" t="inlineStr">
+      <c r="H80" t="inlineStr">
         <is>
           <t>CASE - Visible defect on terminal block surface (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+    <row r="81">
+      <c r="A81" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>NISSEN</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D81" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="E81" t="inlineStr">
         <is>
           <t>Cable Harness</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="F81" t="inlineStr">
         <is>
           <t>VE102-33C</t>
         </is>
       </c>
-      <c r="G46" s="3" t="n">
+      <c r="G81" t="n">
         <v>4</v>
       </c>
-      <c r="H46" s="4" t="inlineStr">
+      <c r="H81" t="inlineStr">
         <is>
           <t>CASE - Cable Harness function test failed (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="82">
+      <c r="A82" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B82" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F82" t="inlineStr">
         <is>
           <t>PL-2019</t>
         </is>
       </c>
-      <c r="G47" s="3" t="n">
+      <c r="G82" t="n">
         <v>12</v>
       </c>
-      <c r="H47" s="4" t="inlineStr">
+      <c r="H82" t="inlineStr">
         <is>
           <t>CASE - Color mismatch vs Pantone reference (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+    <row r="83">
+      <c r="A83" t="inlineStr">
         <is>
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D83" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E83" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F83" t="inlineStr">
         <is>
           <t>RB-200</t>
         </is>
       </c>
-      <c r="G48" s="3" t="n">
+      <c r="G83" t="n">
         <v>23</v>
       </c>
-      <c r="H48" s="3" t="inlineStr">
+      <c r="H83" t="inlineStr">
         <is>
           <t>Surface scratch on terminal block</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+    <row r="84">
+      <c r="A84" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C49" s="2" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>COLOR NG</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E84" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="F84" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G49" s="3" t="n">
+      <c r="G84" t="n">
         <v>2</v>
       </c>
-      <c r="H49" s="3" t="inlineStr">
+      <c r="H84" t="inlineStr">
         <is>
           <t>Terminal Block leak detected at joint</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+    <row r="85">
+      <c r="A85" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D85" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E50" s="3" t="inlineStr">
+      <c r="E85" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="F85" t="inlineStr">
         <is>
           <t>VE101-22A</t>
         </is>
       </c>
-      <c r="G50" s="3" t="n">
+      <c r="G85" t="n">
         <v>6</v>
       </c>
-      <c r="H50" s="4" t="inlineStr">
+      <c r="H85" t="inlineStr">
         <is>
           <t>CASE - Battery Cell Holder dimension out of spec by 0.2mm (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+    <row r="86">
+      <c r="A86" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>NISSEN</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>COLOR NG</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F86" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G51" s="3" t="n">
+      <c r="G86" t="n">
         <v>12</v>
       </c>
-      <c r="H51" s="3" t="inlineStr">
+      <c r="H86" t="inlineStr">
         <is>
           <t>Gasket Ring function test failed</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+    <row r="87">
+      <c r="A87" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>C.G.</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="D87" t="inlineStr">
         <is>
           <t>SURFACE DEFECT</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
+      <c r="E87" t="inlineStr">
         <is>
           <t>Cover Cap</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="F87" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G52" s="3" t="n">
+      <c r="G87" t="n">
         <v>17</v>
       </c>
-      <c r="H52" s="4" t="inlineStr">
+      <c r="H87" t="inlineStr">
         <is>
           <t>CASE - Visible defect on cover cap surface (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+    <row r="88">
+      <c r="A88" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>PRINTING</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E53" s="3" t="inlineStr">
+      <c r="E88" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
+      <c r="F88" t="inlineStr">
         <is>
           <t>PR-BARCODE</t>
         </is>
       </c>
-      <c r="G53" s="3" t="n">
+      <c r="G88" t="n">
         <v>15</v>
       </c>
-      <c r="H53" s="3" t="inlineStr">
+      <c r="H88" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be PR-LABEL</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
+    <row r="89">
+      <c r="A89" t="inlineStr">
         <is>
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="B89" t="inlineStr">
         <is>
           <t>NISSEN</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
+      <c r="D89" t="inlineStr">
         <is>
           <t>SURFACE DEFECT</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
+      <c r="E89" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="F89" t="inlineStr">
         <is>
           <t>SM-C3</t>
         </is>
       </c>
-      <c r="G54" s="3" t="n">
+      <c r="G89" t="n">
         <v>4</v>
       </c>
-      <c r="H54" s="3" t="inlineStr">
+      <c r="H89" t="inlineStr">
         <is>
           <t>Gasket Ring function test failed</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+    <row r="90">
+      <c r="A90" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D90" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="E90" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F90" t="inlineStr">
         <is>
           <t>PK-001</t>
         </is>
       </c>
-      <c r="G55" s="3" t="n">
+      <c r="G90" t="n">
         <v>14</v>
       </c>
-      <c r="H55" s="3" t="inlineStr">
+      <c r="H90" t="inlineStr">
         <is>
           <t>Surface scratch on battery cell holder</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+    <row r="91">
+      <c r="A91" t="inlineStr">
         <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>SAM NEO</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F91" t="inlineStr">
         <is>
           <t>SM-C3</t>
         </is>
       </c>
-      <c r="G56" s="3" t="n">
+      <c r="G91" t="n">
         <v>22</v>
       </c>
-      <c r="H56" s="3" t="inlineStr">
+      <c r="H91" t="inlineStr">
         <is>
           <t>Battery Cell Holder function test failed</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="92">
+      <c r="A92" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>C.G.</t>
         </is>
       </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr">
+      <c r="F92" t="inlineStr">
         <is>
           <t>PK-002</t>
         </is>
       </c>
-      <c r="G57" s="3" t="n">
+      <c r="G92" t="n">
         <v>21</v>
       </c>
-      <c r="H57" s="4" t="inlineStr">
+      <c r="H92" t="inlineStr">
         <is>
           <t>CASE - Main Board function test failed (lot rejected)</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+    <row r="93">
+      <c r="A93" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>SURFACE DEFECT</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F93" t="inlineStr">
         <is>
           <t>PL-3001</t>
         </is>
       </c>
-      <c r="G58" s="3" t="n">
+      <c r="G93" t="n">
         <v>10</v>
       </c>
-      <c r="H58" s="4" t="inlineStr">
+      <c r="H93" t="inlineStr">
         <is>
           <t>CASE - Wrong part delivered - should be PL-2020 (lot rejected)</t>
         </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>Total Records</t>
-        </is>
-      </c>
-      <c r="B2" s="7" t="n">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Total QTY (PCS)</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="n">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Total CASE</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Date Range</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>2026-08-20 to 2026-09-02</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Unique Suppliers</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>Unique Parts</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data(schema): add Found + Severity columns
New schema (10 columns):
  Date, Found, Supplier, Group Part, Problem Mode,
  Part Name, Part No, Qty, Severity, Comment

Backfill strategy:
- Found: EMPTY (all 92 records) — pending user input, requires
  knowing inspection stage (IN LINE / FINAL / INCOMING / OQA / CUSTOMER)
  which cannot be reliably inferred from existing Comment text
- Severity: heuristic backfill on 92 records:
    CRITICAL (47): CASE/REJECT keywords, LEAK/FUNCTION NG/SAFETY problems
    MAJOR    (36): qty>=50, dimension/mismatch keywords, dimension NG/part mistake
    MINOR    ( 9): everything else (appearance, scratch, etc.)
</commit_message>
<xml_diff>
--- a/QA_Defects_Data.xlsx
+++ b/QA_Defects_Data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H93"/>
+  <dimension ref="A1:J93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,35 +424,45 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Found</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Supplier</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Group Part</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Problem Mode</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Part Name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Part No</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
         <is>
           <t>Comment</t>
         </is>
@@ -464,35 +474,40 @@
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>GASKET RING</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>PAR-001</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>120</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>Surface scratch found on outer diameter</t>
         </is>
@@ -504,35 +519,40 @@
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>PIPE CONNECTOR</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>VE100-15B</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>5</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>Wrong part shipped - mismatch with PO</t>
         </is>
@@ -544,35 +564,40 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>ELBOW PIPE 1/2</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>VE101-22A</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>50</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>Dimensional out of spec by 0.2mm</t>
         </is>
@@ -584,35 +609,40 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>O-RING SEAL</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>AC2019-A</t>
         </is>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>2</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>Color mismatch with sample</t>
         </is>
@@ -624,35 +654,40 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>KSV</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>HOSE CLAMP</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>AC2020-B</t>
         </is>
       </c>
-      <c r="G6" t="n">
+      <c r="H6" t="n">
         <v>5</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>Color mismatch with sample</t>
         </is>
@@ -664,35 +699,40 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>GASKET RING</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>PAR-001</t>
         </is>
       </c>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>5</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Color mismatch with sample</t>
         </is>
@@ -704,35 +744,40 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>O-RING SEAL</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>AC2019-A</t>
         </is>
       </c>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>50</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>Surface scratch found on outer diameter</t>
         </is>
@@ -744,35 +789,40 @@
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>VALVE BODY</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>PAR-002</t>
         </is>
       </c>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>8</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>Dimensional out of spec by 0.2mm</t>
         </is>
@@ -784,35 +834,40 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>C.G.</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>PIPE CONNECTOR</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>VE100-15B</t>
         </is>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>120</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>Color mismatch with sample</t>
         </is>
@@ -824,35 +879,40 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>HOSE CLAMP</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>AC2020-B</t>
         </is>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>120</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>Color mismatch with sample</t>
         </is>
@@ -864,35 +924,40 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>VALVE BODY</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>PAR-002</t>
         </is>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>2</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>Function test failed - leakage detected</t>
         </is>
@@ -904,35 +969,40 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>HEAT SHRINK</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>NS-CHEM-002</t>
         </is>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>120</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>Dimensional out of spec by 0.2mm</t>
         </is>
@@ -944,35 +1014,40 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>TERMINAL BLOCK</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>NS-CHEM-001</t>
         </is>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>50</v>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>Surface contamination visible</t>
         </is>
@@ -984,35 +1059,40 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>PIPE CONNECTOR</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>VE100-15B</t>
         </is>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>1</v>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>Wrong part shipped - mismatch with PO</t>
         </is>
@@ -1024,35 +1104,40 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>NISSEN CHEMITEC</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>GASKET RING</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>PAR-001</t>
         </is>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>3</v>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>Crack visible at weld joint</t>
         </is>
@@ -1064,35 +1149,40 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>PIPE CONNECTOR</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>VE100-15B</t>
         </is>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>8</v>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>Surface scratch found on outer diameter</t>
         </is>
@@ -1104,35 +1194,40 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>VALVE BODY</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>PAR-002</t>
         </is>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>3</v>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>Surface contamination visible</t>
         </is>
@@ -1144,35 +1239,40 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>PIPE CONNECTOR</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>VE100-15B</t>
         </is>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>12</v>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>MINOR</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>Function test failed - leakage detected</t>
         </is>
@@ -1184,35 +1284,40 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>NISSEN CHEMITEC</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>TERMINAL BLOCK</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>NS-CHEM-001</t>
         </is>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>25</v>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>Dimensional out of spec by 0.2mm</t>
         </is>
@@ -1224,35 +1329,40 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>KSV</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>TERMINAL BLOCK</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>VE101-22A</t>
         </is>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>250</v>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
         <is>
           <t>Major defect - entire batch rejected</t>
         </is>
@@ -1264,35 +1374,40 @@
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>PIPE CONNECTOR</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>VE100-15B</t>
         </is>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>1</v>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>Dimensional out of spec by 0.2mm</t>
         </is>
@@ -1304,35 +1419,40 @@
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>HOSE CLAMP</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>AC2020-B</t>
         </is>
       </c>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>3</v>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>Dimensional out of spec by 0.2mm</t>
         </is>
@@ -1344,35 +1464,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>GASKET RING</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>PAR-001</t>
         </is>
       </c>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>1</v>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
         <is>
           <t>Surface scratch found on outer diameter</t>
         </is>
@@ -1384,35 +1509,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>TERMINAL BLOCK</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>NS-CHEM-001</t>
         </is>
       </c>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>1</v>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>Surface contamination visible</t>
         </is>
@@ -1424,35 +1554,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>TERMINAL BLOCK</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>NS-CHEM-001</t>
         </is>
       </c>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
         <v>1</v>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>Surface contamination visible</t>
         </is>
@@ -1464,35 +1599,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>HOSE CLAMP</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>AC2020-B</t>
         </is>
       </c>
-      <c r="G27" t="n">
+      <c r="H27" t="n">
         <v>1</v>
       </c>
-      <c r="H27" t="inlineStr">
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>MINOR</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>Surface contamination visible</t>
         </is>
@@ -1504,35 +1644,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>C.G.</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>HOSE CLAMP</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>AC2020-B</t>
         </is>
       </c>
-      <c r="G28" t="n">
+      <c r="H28" t="n">
         <v>3</v>
       </c>
-      <c r="H28" t="inlineStr">
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
         <is>
           <t>Crack visible at weld joint</t>
         </is>
@@ -1544,35 +1689,40 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>NISSEN CHEMITEC</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>TERMINAL BLOCK</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>NS-CHEM-001</t>
         </is>
       </c>
-      <c r="G29" t="n">
+      <c r="H29" t="n">
         <v>2</v>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
         <is>
           <t>Dimensional out of spec by 0.2mm</t>
         </is>
@@ -1584,35 +1734,40 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>C.G.</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>GASKET RING</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>PAR-001</t>
         </is>
       </c>
-      <c r="G30" t="n">
+      <c r="H30" t="n">
         <v>1</v>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>MINOR</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
         <is>
           <t>Function test failed - leakage detected</t>
         </is>
@@ -1624,35 +1779,40 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>KSV</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>ELBOW PIPE 1/2</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>VE101-22A</t>
         </is>
       </c>
-      <c r="G31" t="n">
+      <c r="H31" t="n">
         <v>1</v>
       </c>
-      <c r="H31" t="inlineStr">
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
         <is>
           <t>Function test failed - leakage detected</t>
         </is>
@@ -1664,35 +1824,40 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>HEAT SHRINK</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>NS-CHEM-002</t>
         </is>
       </c>
-      <c r="G32" t="n">
+      <c r="H32" t="n">
         <v>25</v>
       </c>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
         <is>
           <t>Crack visible at weld joint</t>
         </is>
@@ -1704,35 +1869,40 @@
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>C.G.</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>VALVE BODY</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>PAR-002</t>
         </is>
       </c>
-      <c r="G33" t="n">
+      <c r="H33" t="n">
         <v>50</v>
       </c>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
         <is>
           <t>Surface scratch found on outer diameter</t>
         </is>
@@ -1744,35 +1914,40 @@
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>HEAT SHRINK</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>NS-CHEM-002</t>
         </is>
       </c>
-      <c r="G34" t="n">
+      <c r="H34" t="n">
         <v>2</v>
       </c>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>Crack visible at weld joint</t>
         </is>
@@ -1784,35 +1959,40 @@
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>HOSE CLAMP</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>AC2020-B</t>
         </is>
       </c>
-      <c r="G35" t="n">
+      <c r="H35" t="n">
         <v>120</v>
       </c>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t>Surface scratch found on outer diameter</t>
         </is>
@@ -1824,35 +2004,40 @@
           <t>2026-08-19 00:00:00</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>HOSE CLAMP</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>AC2020-B</t>
         </is>
       </c>
-      <c r="G36" t="n">
+      <c r="H36" t="n">
         <v>1000</v>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>Surface scratch found on outer diameter</t>
         </is>
@@ -1864,35 +2049,40 @@
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>NISSEN</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>SL-50</t>
         </is>
       </c>
-      <c r="G37" t="n">
+      <c r="H37" t="n">
         <v>5</v>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be SL-75</t>
         </is>
@@ -1904,35 +2094,40 @@
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>VE102-33C</t>
         </is>
       </c>
-      <c r="G38" t="n">
+      <c r="H38" t="n">
         <v>2</v>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
         <is>
           <t>Battery Cell Holder dimension out of spec by 0.2mm</t>
         </is>
@@ -1944,35 +2139,40 @@
           <t>2026-09-02</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>PL-2020</t>
         </is>
       </c>
-      <c r="G39" t="n">
+      <c r="H39" t="n">
         <v>11</v>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
         <is>
           <t>CASE - LED Indicator dimension out of spec by 0.2mm (lot rejected)</t>
         </is>
@@ -1984,35 +2184,40 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>KSV</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>SM-A1</t>
         </is>
       </c>
-      <c r="G40" t="n">
+      <c r="H40" t="n">
         <v>6</v>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
         <is>
           <t>Color mismatch vs Pantone reference</t>
         </is>
@@ -2024,35 +2229,40 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>RB-100</t>
         </is>
       </c>
-      <c r="G41" t="n">
+      <c r="H41" t="n">
         <v>16</v>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
         <is>
           <t>Surface scratch on gasket ring</t>
         </is>
@@ -2064,35 +2274,40 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>APT</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="E42" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="F42" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G42" t="n">
+      <c r="H42" t="n">
         <v>8</v>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
         <is>
           <t>CASE - Color mismatch vs Pantone reference (lot rejected)</t>
         </is>
@@ -2104,35 +2319,40 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>PL-2020</t>
         </is>
       </c>
-      <c r="G43" t="n">
+      <c r="H43" t="n">
         <v>23</v>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
         <is>
           <t>Visible defect on terminal block surface</t>
         </is>
@@ -2144,35 +2364,40 @@
           <t>2026-09-01</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="E44" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="F44" t="inlineStr">
         <is>
           <t>Cover Cap</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>P-101</t>
         </is>
       </c>
-      <c r="G44" t="n">
+      <c r="H44" t="n">
         <v>24</v>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
         <is>
           <t>CASE - Cover Cap function test failed (lot rejected)</t>
         </is>
@@ -2184,35 +2409,40 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>PK-001</t>
         </is>
       </c>
-      <c r="G45" t="n">
+      <c r="H45" t="n">
         <v>5</v>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be PK-001</t>
         </is>
@@ -2224,35 +2454,40 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="F46" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>PK-002</t>
         </is>
       </c>
-      <c r="G46" t="n">
+      <c r="H46" t="n">
         <v>4</v>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
         <is>
           <t>Main Board dimension out of spec by 0.2mm</t>
         </is>
@@ -2264,35 +2499,40 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="F47" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>PK-001</t>
         </is>
       </c>
-      <c r="G47" t="n">
+      <c r="H47" t="n">
         <v>17</v>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
         <is>
           <t>CASE - Gasket Ring dimension out of spec by 0.2mm (lot rejected)</t>
         </is>
@@ -2304,35 +2544,40 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="F48" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>RB-100</t>
         </is>
       </c>
-      <c r="G48" t="n">
+      <c r="H48" t="n">
         <v>17</v>
       </c>
-      <c r="H48" t="inlineStr">
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
         <is>
           <t>Surface scratch on switch button</t>
         </is>
@@ -2344,35 +2589,40 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>VE103-44D</t>
         </is>
       </c>
-      <c r="G49" t="n">
+      <c r="H49" t="n">
         <v>20</v>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be VE100-15C</t>
         </is>
@@ -2384,35 +2634,40 @@
           <t>2026-08-31</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>VE100-15C</t>
         </is>
       </c>
-      <c r="G50" t="n">
+      <c r="H50" t="n">
         <v>25</v>
       </c>
-      <c r="H50" t="inlineStr">
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
         <is>
           <t>Visible defect on led indicator surface</t>
         </is>
@@ -2424,35 +2679,40 @@
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>VE100-15C</t>
         </is>
       </c>
-      <c r="G51" t="n">
+      <c r="H51" t="n">
         <v>6</v>
       </c>
-      <c r="H51" t="inlineStr">
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
         <is>
           <t>Visible defect on switch button surface</t>
         </is>
@@ -2464,35 +2724,40 @@
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="C52" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>SURFACE DEFECT</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>RM-A</t>
         </is>
       </c>
-      <c r="G52" t="n">
+      <c r="H52" t="n">
         <v>19</v>
       </c>
-      <c r="H52" t="inlineStr">
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>MINOR</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>Surface scratch on switch button</t>
         </is>
@@ -2504,35 +2769,40 @@
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>PRINTING</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>PR-BARCODE</t>
         </is>
       </c>
-      <c r="G53" t="n">
+      <c r="H53" t="n">
         <v>4</v>
       </c>
-      <c r="H53" t="inlineStr">
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
         <is>
           <t>LED Indicator leak detected at joint</t>
         </is>
@@ -2544,35 +2814,40 @@
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>VE103-44D</t>
         </is>
       </c>
-      <c r="G54" t="n">
+      <c r="H54" t="n">
         <v>23</v>
       </c>
-      <c r="H54" t="inlineStr">
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
         <is>
           <t>Gasket Ring dimension out of spec by 0.2mm</t>
         </is>
@@ -2584,35 +2859,40 @@
           <t>2026-08-30</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="F55" t="inlineStr">
         <is>
           <t>Cable Harness</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>RB-200</t>
         </is>
       </c>
-      <c r="G55" t="n">
+      <c r="H55" t="n">
         <v>9</v>
       </c>
-      <c r="H55" t="inlineStr">
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
         <is>
           <t>Color mismatch vs Pantone reference</t>
         </is>
@@ -2624,35 +2904,40 @@
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>SAM NEO</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="F56" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>RM-B</t>
         </is>
       </c>
-      <c r="G56" t="n">
+      <c r="H56" t="n">
         <v>2</v>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
         <is>
           <t>CASE - Gasket Ring leak detected at joint (lot rejected)</t>
         </is>
@@ -2664,35 +2949,40 @@
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>SM-A1</t>
         </is>
       </c>
-      <c r="G57" t="n">
+      <c r="H57" t="n">
         <v>14</v>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>MINOR</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
         <is>
           <t>Switch Button function test failed</t>
         </is>
@@ -2704,35 +2994,40 @@
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>Cover Cap</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>PL-2020</t>
         </is>
       </c>
-      <c r="G58" t="n">
+      <c r="H58" t="n">
         <v>15</v>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
         <is>
           <t>Cover Cap function test failed</t>
         </is>
@@ -2744,35 +3039,40 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>SAM NEO</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>COLOR NG</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>VE101-22A</t>
         </is>
       </c>
-      <c r="G59" t="n">
+      <c r="H59" t="n">
         <v>22</v>
       </c>
-      <c r="H59" t="inlineStr">
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be VE102-33C</t>
         </is>
@@ -2784,35 +3084,40 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="E60" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="F60" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="G60" t="inlineStr">
         <is>
           <t>PK-001</t>
         </is>
       </c>
-      <c r="G60" t="n">
+      <c r="H60" t="n">
         <v>24</v>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be PK-001</t>
         </is>
@@ -2824,35 +3129,40 @@
           <t>2026-08-28</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>KSV</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>PRINTING</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="G61" t="inlineStr">
         <is>
           <t>PR-LABEL</t>
         </is>
       </c>
-      <c r="G61" t="n">
+      <c r="H61" t="n">
         <v>22</v>
       </c>
-      <c r="H61" t="inlineStr">
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be PR-LABEL</t>
         </is>
@@ -2864,35 +3174,40 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="C62" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="D62" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="F62" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G62" t="n">
+      <c r="H62" t="n">
         <v>12</v>
       </c>
-      <c r="H62" t="inlineStr">
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
         <is>
           <t>Visible defect on terminal block surface</t>
         </is>
@@ -2904,35 +3219,40 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t>SM-A1</t>
         </is>
       </c>
-      <c r="G63" t="n">
+      <c r="H63" t="n">
         <v>24</v>
       </c>
-      <c r="H63" t="inlineStr">
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
         <is>
           <t>CASE - Main Board dimension out of spec by 0.2mm (lot rejected)</t>
         </is>
@@ -2944,35 +3264,40 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="G64" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G64" t="n">
+      <c r="H64" t="n">
         <v>16</v>
       </c>
-      <c r="H64" t="inlineStr">
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
         <is>
           <t>CASE - Battery Cell Holder leak detected at joint (lot rejected)</t>
         </is>
@@ -2984,35 +3309,40 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="C65" t="inlineStr">
         <is>
           <t>C.G.</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="D65" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="F65" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="G65" t="inlineStr">
         <is>
           <t>RM-A</t>
         </is>
       </c>
-      <c r="G65" t="n">
+      <c r="H65" t="n">
         <v>11</v>
       </c>
-      <c r="H65" t="inlineStr">
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be RM-B</t>
         </is>
@@ -3024,35 +3354,40 @@
           <t>2026-08-27</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="C66" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="G66" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G66" t="n">
+      <c r="H66" t="n">
         <v>17</v>
       </c>
-      <c r="H66" t="inlineStr">
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be SL-75</t>
         </is>
@@ -3064,35 +3399,40 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
+      <c r="C67" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C67" t="inlineStr">
+      <c r="D67" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="E67" t="inlineStr">
         <is>
           <t>COLOR NG</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr">
+      <c r="F67" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="G67" t="inlineStr">
         <is>
           <t>PK-002</t>
         </is>
       </c>
-      <c r="G67" t="n">
+      <c r="H67" t="n">
         <v>4</v>
       </c>
-      <c r="H67" t="inlineStr">
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
         <is>
           <t>Color mismatch vs Pantone reference</t>
         </is>
@@ -3104,35 +3444,40 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>TECHNO ASSOCIATE</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="D68" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="E68" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="F68" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="G68" t="inlineStr">
         <is>
           <t>VE100-15C</t>
         </is>
       </c>
-      <c r="G68" t="n">
+      <c r="H68" t="n">
         <v>4</v>
       </c>
-      <c r="H68" t="inlineStr">
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
         <is>
           <t>CASE - Color mismatch vs Pantone reference (lot rejected)</t>
         </is>
@@ -3144,35 +3489,40 @@
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t>SAM NEO</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="D69" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr">
+      <c r="F69" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>P-330</t>
         </is>
       </c>
-      <c r="G69" t="n">
+      <c r="H69" t="n">
         <v>7</v>
       </c>
-      <c r="H69" t="inlineStr">
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
         <is>
           <t>Visible defect on battery cell holder surface</t>
         </is>
@@ -3184,35 +3534,40 @@
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="C70" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>RM-A</t>
         </is>
       </c>
-      <c r="G70" t="n">
+      <c r="H70" t="n">
         <v>22</v>
       </c>
-      <c r="H70" t="inlineStr">
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be RM-A</t>
         </is>
@@ -3224,35 +3579,40 @@
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="E71" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="G71" t="inlineStr">
         <is>
           <t>P-330</t>
         </is>
       </c>
-      <c r="G71" t="n">
+      <c r="H71" t="n">
         <v>10</v>
       </c>
-      <c r="H71" t="inlineStr">
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
         <is>
           <t>Main Board leak detected at joint</t>
         </is>
@@ -3264,35 +3624,40 @@
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="C72" t="inlineStr">
         <is>
           <t>NISSEN</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="D72" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>Cover Cap</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="G72" t="inlineStr">
         <is>
           <t>RB-100</t>
         </is>
       </c>
-      <c r="G72" t="n">
+      <c r="H72" t="n">
         <v>12</v>
       </c>
-      <c r="H72" t="inlineStr">
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
         <is>
           <t>Visible defect on cover cap surface</t>
         </is>
@@ -3304,35 +3669,40 @@
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>PARADISE</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="G73" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G73" t="n">
+      <c r="H73" t="n">
         <v>14</v>
       </c>
-      <c r="H73" t="inlineStr">
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
         <is>
           <t>CASE - Terminal Block dimension out of spec by 0.2mm (lot rejected)</t>
         </is>
@@ -3344,35 +3714,40 @@
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>AKUSAN</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>PRINTING</t>
         </is>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>LED Indicator</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="G74" t="inlineStr">
         <is>
           <t>PR-BARCODE</t>
         </is>
       </c>
-      <c r="G74" t="n">
+      <c r="H74" t="n">
         <v>6</v>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be PR-LABEL</t>
         </is>
@@ -3384,35 +3759,40 @@
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="F75" t="inlineStr">
         <is>
           <t>Switch Button</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="G75" t="inlineStr">
         <is>
           <t>RB-200</t>
         </is>
       </c>
-      <c r="G75" t="n">
+      <c r="H75" t="n">
         <v>13</v>
       </c>
-      <c r="H75" t="inlineStr">
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
         <is>
           <t>CASE - Surface scratch on switch button (lot rejected)</t>
         </is>
@@ -3424,35 +3804,40 @@
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="C76" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>PIPING</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>Cable Harness</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="G76" t="inlineStr">
         <is>
           <t>P-205</t>
         </is>
       </c>
-      <c r="G76" t="n">
+      <c r="H76" t="n">
         <v>3</v>
       </c>
-      <c r="H76" t="inlineStr">
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
         <is>
           <t>Surface scratch on cable harness</t>
         </is>
@@ -3464,35 +3849,40 @@
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="D77" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>FUNCTION NG</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>Cable Harness</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="G77" t="inlineStr">
         <is>
           <t>PK-001</t>
         </is>
       </c>
-      <c r="G77" t="n">
+      <c r="H77" t="n">
         <v>4</v>
       </c>
-      <c r="H77" t="inlineStr">
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
         <is>
           <t>Visible defect on cable harness surface</t>
         </is>
@@ -3504,35 +3894,40 @@
           <t>2026-08-24</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="D78" t="inlineStr">
         <is>
           <t>RAW MATERIAL</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>COLOR NG</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr">
+      <c r="F78" t="inlineStr">
         <is>
           <t>Cable Harness</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="G78" t="inlineStr">
         <is>
           <t>RM-A</t>
         </is>
       </c>
-      <c r="G78" t="n">
+      <c r="H78" t="n">
         <v>22</v>
       </c>
-      <c r="H78" t="inlineStr">
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be RM-A</t>
         </is>
@@ -3544,35 +3939,40 @@
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="E79" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="F79" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="G79" t="inlineStr">
         <is>
           <t>PL-2019</t>
         </is>
       </c>
-      <c r="G79" t="n">
+      <c r="H79" t="n">
         <v>19</v>
       </c>
-      <c r="H79" t="inlineStr">
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
         <is>
           <t>Color mismatch vs Pantone reference</t>
         </is>
@@ -3584,35 +3984,40 @@
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
+      <c r="C80" t="inlineStr">
         <is>
           <t>BTD</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
+      <c r="D80" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="E80" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr">
+      <c r="F80" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="G80" t="inlineStr">
         <is>
           <t>VE101-22A</t>
         </is>
       </c>
-      <c r="G80" t="n">
+      <c r="H80" t="n">
         <v>13</v>
       </c>
-      <c r="H80" t="inlineStr">
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
         <is>
           <t>CASE - Visible defect on terminal block surface (lot rejected)</t>
         </is>
@@ -3624,35 +4029,40 @@
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>NISSEN</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="D81" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="E81" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="F81" t="inlineStr">
         <is>
           <t>Cable Harness</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="G81" t="inlineStr">
         <is>
           <t>VE102-33C</t>
         </is>
       </c>
-      <c r="G81" t="n">
+      <c r="H81" t="n">
         <v>4</v>
       </c>
-      <c r="H81" t="inlineStr">
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
         <is>
           <t>CASE - Cable Harness function test failed (lot rejected)</t>
         </is>
@@ -3664,35 +4074,40 @@
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="C82" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="D82" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="E82" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr">
+      <c r="F82" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="G82" t="inlineStr">
         <is>
           <t>PL-2019</t>
         </is>
       </c>
-      <c r="G82" t="n">
+      <c r="H82" t="n">
         <v>12</v>
       </c>
-      <c r="H82" t="inlineStr">
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
         <is>
           <t>CASE - Color mismatch vs Pantone reference (lot rejected)</t>
         </is>
@@ -3704,35 +4119,40 @@
           <t>2026-08-23</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>TTS PLASTIC</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="D83" t="inlineStr">
         <is>
           <t>RUBBER</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="E83" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="F83" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="G83" t="inlineStr">
         <is>
           <t>RB-200</t>
         </is>
       </c>
-      <c r="G83" t="n">
+      <c r="H83" t="n">
         <v>23</v>
       </c>
-      <c r="H83" t="inlineStr">
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
         <is>
           <t>Surface scratch on terminal block</t>
         </is>
@@ -3744,35 +4164,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="E84" t="inlineStr">
         <is>
           <t>COLOR NG</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="F84" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="G84" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G84" t="n">
+      <c r="H84" t="n">
         <v>2</v>
       </c>
-      <c r="H84" t="inlineStr">
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>MINOR</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
         <is>
           <t>Terminal Block leak detected at joint</t>
         </is>
@@ -3784,35 +4209,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>SUPERFAST</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="D85" t="inlineStr">
         <is>
           <t>ELECTRIC &amp; ELEC.</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="E85" t="inlineStr">
         <is>
           <t>PART MISTAKE</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="F85" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F85" t="inlineStr">
+      <c r="G85" t="inlineStr">
         <is>
           <t>VE101-22A</t>
         </is>
       </c>
-      <c r="G85" t="n">
+      <c r="H85" t="n">
         <v>6</v>
       </c>
-      <c r="H85" t="inlineStr">
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
         <is>
           <t>CASE - Battery Cell Holder dimension out of spec by 0.2mm (lot rejected)</t>
         </is>
@@ -3824,35 +4254,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>NISSEN</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>COLOR NG</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr">
+      <c r="F86" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr">
+      <c r="G86" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G86" t="n">
+      <c r="H86" t="n">
         <v>12</v>
       </c>
-      <c r="H86" t="inlineStr">
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>MINOR</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
         <is>
           <t>Gasket Ring function test failed</t>
         </is>
@@ -3864,35 +4299,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>C.G.</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="D87" t="inlineStr">
         <is>
           <t>SEALING</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="E87" t="inlineStr">
         <is>
           <t>SURFACE DEFECT</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="F87" t="inlineStr">
         <is>
           <t>Cover Cap</t>
         </is>
       </c>
-      <c r="F87" t="inlineStr">
+      <c r="G87" t="inlineStr">
         <is>
           <t>SL-75</t>
         </is>
       </c>
-      <c r="G87" t="n">
+      <c r="H87" t="n">
         <v>17</v>
       </c>
-      <c r="H87" t="inlineStr">
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
         <is>
           <t>CASE - Visible defect on cover cap surface (lot rejected)</t>
         </is>
@@ -3904,35 +4344,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>PRINTING</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="E88" t="inlineStr">
         <is>
           <t>DIMENSION NG</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr">
+      <c r="F88" t="inlineStr">
         <is>
           <t>Terminal Block</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr">
+      <c r="G88" t="inlineStr">
         <is>
           <t>PR-BARCODE</t>
         </is>
       </c>
-      <c r="G88" t="n">
+      <c r="H88" t="n">
         <v>15</v>
       </c>
-      <c r="H88" t="inlineStr">
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>MAJOR</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
         <is>
           <t>Wrong part delivered - should be PR-LABEL</t>
         </is>
@@ -3944,35 +4389,40 @@
           <t>2026-08-22</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>NISSEN</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="D89" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="E89" t="inlineStr">
         <is>
           <t>SURFACE DEFECT</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="F89" t="inlineStr">
         <is>
           <t>Gasket Ring</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="G89" t="inlineStr">
         <is>
           <t>SM-C3</t>
         </is>
       </c>
-      <c r="G89" t="n">
+      <c r="H89" t="n">
         <v>4</v>
       </c>
-      <c r="H89" t="inlineStr">
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>MINOR</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
         <is>
           <t>Gasket Ring function test failed</t>
         </is>
@@ -3984,35 +4434,40 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>DEM</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="D90" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="E90" t="inlineStr">
         <is>
           <t>LEAK</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr">
+      <c r="F90" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F90" t="inlineStr">
+      <c r="G90" t="inlineStr">
         <is>
           <t>PK-001</t>
         </is>
       </c>
-      <c r="G90" t="n">
+      <c r="H90" t="n">
         <v>14</v>
       </c>
-      <c r="H90" t="inlineStr">
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
         <is>
           <t>Surface scratch on battery cell holder</t>
         </is>
@@ -4024,35 +4479,40 @@
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>SAM NEO</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>SHEET METAL</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
+      <c r="F91" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F91" t="inlineStr">
+      <c r="G91" t="inlineStr">
         <is>
           <t>SM-C3</t>
         </is>
       </c>
-      <c r="G91" t="n">
+      <c r="H91" t="n">
         <v>22</v>
       </c>
-      <c r="H91" t="inlineStr">
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>MINOR</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
         <is>
           <t>Battery Cell Holder function test failed</t>
         </is>
@@ -4064,35 +4524,40 @@
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>C.G.</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>PACKING</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>APPEARANCE NG</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
+      <c r="F92" t="inlineStr">
         <is>
           <t>Main Board</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr">
+      <c r="G92" t="inlineStr">
         <is>
           <t>PK-002</t>
         </is>
       </c>
-      <c r="G92" t="n">
+      <c r="H92" t="n">
         <v>21</v>
       </c>
-      <c r="H92" t="inlineStr">
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
         <is>
           <t>CASE - Main Board function test failed (lot rejected)</t>
         </is>
@@ -4104,35 +4569,40 @@
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>SAMBO</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>PLASTIC</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>SURFACE DEFECT</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
+      <c r="F93" t="inlineStr">
         <is>
           <t>Battery Cell Holder</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr">
+      <c r="G93" t="inlineStr">
         <is>
           <t>PL-3001</t>
         </is>
       </c>
-      <c r="G93" t="n">
+      <c r="H93" t="n">
         <v>10</v>
       </c>
-      <c r="H93" t="inlineStr">
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
         <is>
           <t>CASE - Wrong part delivered - should be PL-2020 (lot rejected)</t>
         </is>

</xml_diff>